<commit_message>
P1/L1.1: record author review and update novelty matrix
</commit_message>
<xml_diff>
--- a/notes/01_literature/novelty_matrix.xlsx
+++ b/notes/01_literature/novelty_matrix.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paper Breakdown" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IRTF NDT Architecture 2026" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AoI Survey 2020" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stale Link State 2001" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OpenTwin 2026" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remote Inference 2024" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conformal Tutorial 2022" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Novelty Matrix" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Papers Comparison" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Paper Breakdown" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="IRTF NDT Architecture 2026" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="AoI Survey 2020" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Stale Link State 2001" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="OpenTwin 2026" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Remote Inference 2024" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Conformal Tutorial 2022" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Novelty Matrix" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="All Papers Comparison" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="K8" s="35" t="inlineStr">
         <is>
-          <t>Metadata v2 đúng (v1 nộp 23/05/2026, v2 nộp 28/08/2026). v1 có tiêu đề khác và chưa có conformal gate → phải trích rõ arXiv:2605.24662v2. Số liệu mức abstract khớp (false approval thấp hơn budget 0.05–0.30 khoảng 1 bậc; giữ ~40% mức tiết kiệm). Các số chi tiết (14.4–34.9%, 5.89%...) CHƯA kiểm được. Câu "AoI không phải conditioning variable của gate" là SUY LUẬN, cần xác nhận ở Section VI.</t>
+          <t>ĐÃ KIỂM full text arXiv:2605.24662v2: §VI pp.6–7 xác nhận gate đánh giá absolute safety của một candidate action bằng C_t(a) ⊆ S; admission không explicit-condition theo telemetry age và không dùng relative top-2 margin. Temporal drift/freshness vẫn được xử lý bằng online calibration và e-detector (§V–VI). Theorem 3 (§VII-C, p.8) bound joint false-approval frequency trên mọi decision steps, không phải selective risk trên ACCEPT. Các số đã kiểm: KPM error 14.4–34.9% → 2.7–6.5% (§VIII-B, p.9); adaptive calibrator 5.89% (§VIII-C, pp.9–10); giữ khoảng 40.1% achievable energy tại α=0.30 (§VIII-E, pp.10–11). Tác giả xác nhận tự đọc/kiểm ngày 2026-09-23; xem opentwin_2026_v2.md.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
P1/L1.2: update novelty synthesis and B6 validation
</commit_message>
<xml_diff>
--- a/notes/01_literature/novelty_matrix.xlsx
+++ b/notes/01_literature/novelty_matrix.xlsx
@@ -13,14 +13,16 @@
     <sheet name="Novelty Matrix" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="All Papers Comparison" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Novelty Matrix'!$A$1:$L$34</definedName>
+  </definedNames>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -66,8 +68,18 @@
       <color rgb="FF1F1F1F"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -124,6 +136,26 @@
         <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF3F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4F8FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border/>
@@ -132,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -311,6 +343,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2112,7 +2159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="54" min="1" max="1"/>
@@ -2126,6 +2173,7 @@
     <col width="30" customWidth="1" style="54" min="9" max="9"/>
     <col width="46" customWidth="1" style="54" min="10" max="10"/>
     <col width="52" customWidth="1" style="54" min="11" max="11"/>
+    <col width="42" customWidth="1" style="54" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="54">
@@ -2184,6 +2232,11 @@
           <t>Kiểm chứng &amp; ưu tiên đọc (cập nhật 23/09/2026)</t>
         </is>
       </c>
+      <c r="L1" s="82" t="inlineStr">
+        <is>
+          <t>Đã kiểm full text (ngày, §)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="134.5" customHeight="1" s="54">
       <c r="A2" s="35" t="inlineStr">
@@ -2241,6 +2294,11 @@
           <t>Đã kiểm với full text (arXiv 2205.14206); metadata đúng: IEEE Commun. Mag. 60(11):22–27, 2022. Bổ sung: tập test chỉ 500 mẫu trên topology 50–300 node. Inference RouteNet-E ≈6.47 s, chậm hơn QT (≈5.1 s) và RNN (≈0.16 s); chỉ nhanh hơn nhiều so với OMNeT++ (≈3h39m). Routing optimization chỉ đánh giá trên 1 topology 25 node, so với shortest path ban đầu. Challenge "uncertainty" gợi ý BNN hoặc kiểm thử vùng vận hành an toàn; paper không tách explainability thành challenge riêng.</t>
         </is>
       </c>
+      <c r="L2" s="35" t="inlineStr">
+        <is>
+          <t>Đã kiểm toàn văn arXiv:2205.14206; ngày 2026-09-23; § case study/evaluation (cột K)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="47.5" customHeight="1" s="54">
       <c r="A3" s="35" t="inlineStr">
@@ -2298,6 +2356,11 @@
           <t>Đã kiểm (datatracker): draft-13, 01/07/2026, đúng tiêu đề. Draft đã qua RG last call nhưng vẫn phải trích dưới dạng "work in progress".</t>
         </is>
       </c>
+      <c r="L3" s="35" t="inlineStr">
+        <is>
+          <t>Chưa xác nhận mức kiểm full text; xem cột K</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="33" customHeight="1" s="54">
       <c r="A4" s="35" t="inlineStr">
@@ -2355,6 +2418,11 @@
           <t>SỬA METADATA: trích bản journal IEEE JSAC 39(5):1183–1210, 05/2021 thay cho arXiv 2020.</t>
         </is>
       </c>
+      <c r="L4" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; mới metadata/abstract, 2026-09-23</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="120" customHeight="1" s="54">
       <c r="A5" s="35" t="inlineStr">
@@ -2412,6 +2480,11 @@
           <t>Metadata đúng (IEEE/ACM ToN 9(2):162–176, 04/2001). Mới kiểm được abstract; các key findings chi tiết cần tự đối chiếu full text. SỬA KHÁI NIỆM: không ghi "không dùng margin". Paper khuyến nghị chỉnh độ thô của link-cost theo độ thiếu chính xác của link-state, tức ý tưởng margin ở mức thiết kế tĩnh. Khác biệt của DT4N: dùng margin để gate TỪNG quyết định và điều kiện hóa theo age.</t>
         </is>
       </c>
+      <c r="L5" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; mới metadata/abstract, 2026-09-23</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="62" customHeight="1" s="54">
       <c r="A6" s="35" t="inlineStr">
@@ -2469,6 +2542,11 @@
           <t>SỬA METADATA: trích IEEE/ACM ToN 32(5):3824–3839, 2024. Claim cốt lõi đã kiểm (chuỗi gần Markov → error đơn điệu theo AoI; xa Markov → có thể không đơn điệu). Hai con số ~3× và ~8× CHƯA kiểm.</t>
         </is>
       </c>
+      <c r="L6" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; mới metadata/abstract, 2026-09-23</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="47.5" customHeight="1" s="54">
       <c r="A7" s="35" t="inlineStr">
@@ -2526,6 +2604,11 @@
           <t>Không thấy vấn đề. (Có thể đã có bản monograph Foundations &amp; Trends in ML 2023; cần tự kiểm trước khi trích.)</t>
         </is>
       </c>
+      <c r="L7" s="35" t="inlineStr">
+        <is>
+          <t>Chưa xác nhận mức kiểm full text; xem cột K</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="120" customHeight="1" s="54">
       <c r="A8" s="35" t="inlineStr">
@@ -2583,6 +2666,11 @@
           <t>ĐÃ KIỂM full text arXiv:2605.24662v2: §VI pp.6–7 xác nhận gate đánh giá absolute safety của một candidate action bằng C_t(a) ⊆ S; admission không explicit-condition theo telemetry age và không dùng relative top-2 margin. Temporal drift/freshness vẫn được xử lý bằng online calibration và e-detector (§V–VI). Theorem 3 (§VII-C, p.8) bound joint false-approval frequency trên mọi decision steps, không phải selective risk trên ACCEPT. Các số đã kiểm: KPM error 14.4–34.9% → 2.7–6.5% (§VIII-B, p.9); adaptive calibrator 5.89% (§VIII-C, pp.9–10); giữ khoảng 40.1% achievable energy tại α=0.30 (§VIII-E, pp.10–11). Tác giả xác nhận tự đọc/kiểm ngày 2026-09-23; xem opentwin_2026_v2.md.</t>
         </is>
       </c>
+      <c r="L8" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-23; arXiv v2 §V–VIII, đặc biệt §VI–VII-C</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="76.5" customHeight="1" s="54">
       <c r="A9" s="77" t="inlineStr">
@@ -2597,7 +2685,7 @@
       </c>
       <c r="C9" s="77" t="inlineStr">
         <is>
-          <t>Gián tiếp: thông tin trạng thái không chính xác (không đo age riêng)</t>
+          <t>Có state aging trong §I-B: update định kỳ/ngưỡng khiến actual state lệch advertised state; không dùng age làm biến gate</t>
         </is>
       </c>
       <c r="D9" s="77" t="inlineStr">
@@ -2607,12 +2695,12 @@
       </c>
       <c r="E9" s="77" t="inlineStr">
         <is>
-          <t>Có ở dạng xác suất: so sánh xác suất đáp ứng QoS giữa các đường (không dùng best-vs-second margin)</t>
+          <t>Có QoS delay slack ở §IV; không phải best-vs-second path-cost margin trong các § đã kiểm</t>
         </is>
       </c>
       <c r="F9" s="77" t="inlineStr">
         <is>
-          <t>Không (chọn đường tốt nhất dưới bất định, không abstain)</t>
+          <t>Không thấy calibrated ACCEPT/ABSTAIN gate trong §I–V; admission là tiêu chí khác được nêu ngoài phạm vi chính</t>
         </is>
       </c>
       <c r="G9" s="77" t="inlineStr">
@@ -2627,7 +2715,7 @@
       </c>
       <c r="I9" s="77" t="inlineStr">
         <is>
-          <t>Lý thuyết + thuật toán; chi tiết evaluation chưa kiểm</t>
+          <t>Lý thuyết + heuristic cho bandwidth/delay; proof Appendix chưa kiểm hết</t>
         </is>
       </c>
       <c r="J9" s="77" t="inlineStr">
@@ -2637,7 +2725,12 @@
       </c>
       <c r="K9" s="77" t="inlineStr">
         <is>
-          <t>Đã kiểm: abstract + metadata. ƯU TIÊN: BẮT BUỘC ĐỌC (Intro, mô hình bất định, thuật toán).</t>
+          <t>ĐÃ KIỂM PDF toàn văn 14 trang, §I–V và Prop. III.1 ngày 2026-09-23; Appendix/proofs chưa kiểm hết. Note guerin_orda_1999.md.</t>
+        </is>
+      </c>
+      <c r="L9" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-23; PDF §I–V, Proposition III.1; Appendix chưa kiểm hết</t>
         </is>
       </c>
     </row>
@@ -2697,6 +2790,11 @@
           <t>Đã kiểm: chỉ metadata (qua trích dẫn chéo). ƯU TIÊN: CHỈ TRÍCH DẪN.</t>
         </is>
       </c>
+      <c r="L10" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; mới metadata/abstract, 2026-09-23</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="91" customHeight="1" s="54">
       <c r="A11" s="77" t="inlineStr">
@@ -2754,6 +2852,11 @@
           <t>Đã kiểm: chỉ metadata. Mô tả "safety-based" là TRÍ NHỚ, chưa kiểm. ƯU TIÊN: ĐỌC LƯỚT.</t>
         </is>
       </c>
+      <c r="L11" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; mới metadata/abstract, 2026-09-23</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="76.5" customHeight="1" s="54">
       <c r="A12" s="77" t="inlineStr">
@@ -2811,6 +2914,11 @@
           <t>Đã kiểm: abstract + metadata. ƯU TIÊN: BẮT BUỘC TRÍCH, đọc lướt phần kết quả.</t>
         </is>
       </c>
+      <c r="L12" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; mới metadata/abstract, 2026-09-23</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="91" customHeight="1" s="54">
       <c r="A13" s="77" t="inlineStr">
@@ -2868,6 +2976,11 @@
           <t>Đã kiểm: abstract + đoạn đóng góp. ƯU TIÊN: ĐỌC LƯỚT phần setup.</t>
         </is>
       </c>
+      <c r="L13" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; mới metadata/abstract, 2026-09-23</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="91" customHeight="1" s="54">
       <c r="A14" s="77" t="inlineStr">
@@ -2902,12 +3015,12 @@
       </c>
       <c r="G14" s="77" t="inlineStr">
         <is>
-          <t>Có: guarantee theo từng action; thuật toán hữu hạn mẫu dựa trên pinball loss (nối với Gibbs et al. 2025)</t>
+          <t>Có: Theorem 4.3 coverage theo action được chọn dưới exchangeability; Corollary 4.4 utility certificate; khác selective risk|ACCEPT</t>
         </is>
       </c>
       <c r="H14" s="77" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
+          <t>Theorem 4.3 cần exchangeability; time dependence cần xử lý riêng</t>
         </is>
       </c>
       <c r="I14" s="77" t="inlineStr">
@@ -2917,12 +3030,17 @@
       </c>
       <c r="J14" s="77" t="inlineStr">
         <is>
-          <t>Không claim guarantee mới cho "quyết định đã được chọn" (post-selection validity của Phase 22 trùng vấn đề). Dùng/trích framework này; định vị contribution ở phía networking.</t>
+          <t>Không claim selected-action conditional guarantee là mới; không áp Theorem 4.3 cho chuỗi thời gian thiếu exchangeability hoặc đồng nhất action identity với ACCEPT.</t>
         </is>
       </c>
       <c r="K14" s="77" t="inlineStr">
         <is>
-          <t>Đã kiểm: abstract. ƯU TIÊN: BẮT BUỘC ĐỌC (Section 2: formulation).</t>
+          <t>ĐÃ KIỂM arXiv:2606.05551v2 PDF §2, §4, Thm 2.1/4.3, Cor.4.4, 2026-09-23; experiment/proof supplement chưa đọc sâu. Note zhu_2026.md.</t>
+        </is>
+      </c>
+      <c r="L14" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-23; arXiv v2 §2, §4, Thm 2.1/4.3, Cor. 4.4</t>
         </is>
       </c>
     </row>
@@ -2982,6 +3100,11 @@
           <t>Đã kiểm: abstract. ƯU TIÊN: CHỈ TRÍCH DẪN.</t>
         </is>
       </c>
+      <c r="L15" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; mới metadata/abstract, 2026-09-23</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="62" customHeight="1" s="54">
       <c r="A16" s="77" t="inlineStr">
@@ -3039,6 +3162,11 @@
           <t>Đã kiểm: abstract + một đoạn kết quả. ƯU TIÊN: ĐỌC LƯỚT; dùng làm lý do cho baseline.</t>
         </is>
       </c>
+      <c r="L16" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; mới metadata/abstract, 2026-09-23</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="76.5" customHeight="1" s="54">
       <c r="A17" s="77" t="inlineStr">
@@ -3096,6 +3224,11 @@
           <t>Đã kiểm: AoS abstract; AoT chỉ metadata. ƯU TIÊN: CHỈ TRÍCH DẪN.</t>
         </is>
       </c>
+      <c r="L17" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; mới metadata/abstract, 2026-09-23</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="120" customHeight="1" s="54">
       <c r="A18" s="77" t="inlineStr">
@@ -3153,6 +3286,11 @@
           <t>Đã kiểm: abstract (arXiv + trang ScienceDirect). Volume/issue CHƯA kiểm; tên tác giả thứ 2 có hai cách viết trong các nguồn (Linsalata/Lisalata) → kiểm theo DOI. ƯU TIÊN: ĐỌC LƯỚT phần AoI-weighted loss.</t>
         </is>
       </c>
+      <c r="L18" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; mới metadata/abstract, 2026-09-23</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="105.5" customHeight="1" s="54">
       <c r="A19" s="77" t="inlineStr">
@@ -3210,6 +3348,11 @@
           <t>Đã kiểm: metadata qua trích dẫn chéo (arXiv 2605.16176). Nội dung chưa đọc. ƯU TIÊN: chỉ lướt DANH SÁCH THAM KHẢO để snowballing họ D.</t>
         </is>
       </c>
+      <c r="L19" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; mới metadata/abstract, 2026-09-23</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="91" customHeight="1" s="54">
       <c r="A20" s="79" t="inlineStr">
@@ -3267,6 +3410,11 @@
           <t>Đã kiểm: chỉ metadata (qua trích dẫn chéo). ƯU TIÊN: CHỈ TRÍCH DẪN.</t>
         </is>
       </c>
+      <c r="L20" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; mới metadata/abstract, 2026-09-23</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="105.5" customHeight="1" s="54">
       <c r="A21" s="77" t="inlineStr">
@@ -3324,86 +3472,845 @@
           <t>Đã kiểm: abstract (kho lưu trữ Sabancı University). ƯU TIÊN: ĐỌC ABSTRACT, trích dẫn.</t>
         </is>
       </c>
+      <c r="L21" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; mới metadata/abstract, 2026-09-23</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="149" customHeight="1" s="54">
-      <c r="A22" s="35" t="inlineStr">
+      <c r="A22" s="80" t="inlineStr">
+        <is>
+          <t>Attri 2026 — CERT: Certified Route Planning under Drifting Costs</t>
+        </is>
+      </c>
+      <c r="B22" s="77" t="inlineStr">
+        <is>
+          <t>RẤT GẦN — route certificate dưới cost cũ (họ A/B/D)</t>
+        </is>
+      </c>
+      <c r="C22" s="77" t="inlineStr">
+        <is>
+          <t>Có: age theo edge và ρ_e·age trong interval</t>
+        </is>
+      </c>
+      <c r="D22" s="77" t="inlineStr">
+        <is>
+          <t>LB≤OPT≤UB; gap chứng nhận route và hướng paid sensing</t>
+        </is>
+      </c>
+      <c r="E22" s="77" t="inlineStr">
+        <is>
+          <t>Có gap certificate; top-2 estimated margin chưa xác nhận</t>
+        </is>
+      </c>
+      <c r="F22" s="77" t="inlineStr">
+        <is>
+          <t>Có freshness gate cho sum-aware bound; execute conservative incumbent</t>
+        </is>
+      </c>
+      <c r="G22" s="77" t="inlineStr">
+        <is>
+          <t>Non-exchangeable weighted conformal + bound có điều kiện A1–A4; T6 nêu selection</t>
+        </is>
+      </c>
+      <c r="H22" s="77" t="inlineStr">
+        <is>
+          <t>Cost drift bị chặn, residual TV drift bị chặn</t>
+        </is>
+      </c>
+      <c r="I22" s="77" t="inlineStr">
+        <is>
+          <t>Synthetic grids + replay city traffic; §6</t>
+        </is>
+      </c>
+      <c r="J22" s="77" t="inlineStr">
+        <is>
+          <t>KHÔNG claim đầu tiên age-aware conformal route certificate hoặc chứng nhận regret route dưới staleness. Đối chiếu A1–A4, T6, và baseline CERT-style trước DP1.</t>
+        </is>
+      </c>
+      <c r="K22" s="77" t="inlineStr">
+        <is>
+          <t>ĐÃ KIỂM các đoạn §1–7 qua toàn văn hiển thị, một phần Appendix, 2026-09-23; DOI 10.31224/7306; preprint. Note: cert_attri_2026.md. Proof/PDF gốc cần đối chiếu.</t>
+        </is>
+      </c>
+      <c r="L22" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-23; §1–7 và một phần Appendix qua toàn văn hiển thị; PDF/proof chưa kiểm hết</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" s="54">
+      <c r="A23" s="80" t="inlineStr">
+        <is>
+          <t>El Halabi &amp; Brandt 2026 — ACI Under Delayed Feedback</t>
+        </is>
+      </c>
+      <c r="B23" s="77" t="inlineStr">
+        <is>
+          <t>GẦN — delayed-feedback ACI (họ E)</t>
+        </is>
+      </c>
+      <c r="C23" s="77" t="inlineStr">
+        <is>
+          <t>Delay τ của label dự báo, KHÁC telemetry age z</t>
+        </is>
+      </c>
+      <c r="D23" s="77" t="inlineStr">
+        <is>
+          <t>Coverage/interval score của forecast</t>
+        </is>
+      </c>
+      <c r="E23" s="77" t="inlineStr">
+        <is>
+          <t>Không route margin</t>
+        </is>
+      </c>
+      <c r="F23" s="77" t="inlineStr">
+        <is>
+          <t>Không action gate</t>
+        </is>
+      </c>
+      <c r="G23" s="77" t="inlineStr">
+        <is>
+          <t>Cận coverage-frequency có τ; approximate marginal bound</t>
+        </is>
+      </c>
+      <c r="H23" s="77" t="inlineStr">
+        <is>
+          <t>AR(1), GARCH, Markov switching, shifts</t>
+        </is>
+      </c>
+      <c r="I23" s="77" t="inlineStr">
+        <is>
+          <t>Simulation; r=τ/L giảm scatter interval score AR(1) 79% (Table 6)</t>
+        </is>
+      </c>
+      <c r="J23" s="77" t="inlineStr">
+        <is>
+          <t>Không claim delay-to-memory là ý tưởng mới nói chung; tách label delay với telemetry age.</t>
+        </is>
+      </c>
+      <c r="K23" s="77" t="inlineStr">
+        <is>
+          <t>ĐÃ KIỂM arXiv:2609.07251v1 PDF các đoạn §1–4, §7–8, Table 6–7, 2026-09-23; note el_halabi_brandt_2026.md.</t>
+        </is>
+      </c>
+      <c r="L23" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-23; arXiv v1 §1–4, §7–8, Table 6–7</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="48" customHeight="1" s="54">
+      <c r="A24" s="80" t="inlineStr">
+        <is>
+          <t>Hallberg Szabadváry 2024 — multi-step ACI</t>
+        </is>
+      </c>
+      <c r="B24" s="77" t="inlineStr">
+        <is>
+          <t>GẦN — per-horizon online calibration (họ E)</t>
+        </is>
+      </c>
+      <c r="C24" s="77" t="inlineStr">
+        <is>
+          <t>Forecast horizon riêng; không mặc nhiên là telemetry age</t>
+        </is>
+      </c>
+      <c r="D24" s="77" t="inlineStr">
+        <is>
+          <t>Per-horizon forecast coverage</t>
+        </is>
+      </c>
+      <c r="E24" s="77" t="inlineStr">
+        <is>
+          <t>Không decision margin</t>
+        </is>
+      </c>
+      <c r="F24" s="77" t="inlineStr">
+        <is>
+          <t>Không action gate</t>
+        </is>
+      </c>
+      <c r="G24" s="77" t="inlineStr">
+        <is>
+          <t>ACI riêng horizon; Eq.9–10 long-run coverage frequency</t>
+        </is>
+      </c>
+      <c r="H24" s="77" t="inlineStr">
+        <is>
+          <t>Time-series forecast</t>
+        </is>
+      </c>
+      <c r="I24" s="77" t="inlineStr">
+        <is>
+          <t>Victoria electricity demand; h=5, illustrative</t>
+        </is>
+      </c>
+      <c r="J24" s="77" t="inlineStr">
+        <is>
+          <t>Không claim chia ACI theo horizon/age bin là mới; dùng làm baseline per-age ACI có kiểm label timing.</t>
+        </is>
+      </c>
+      <c r="K24" s="77" t="inlineStr">
+        <is>
+          <t>ĐÃ KIỂM PMLR 230:250–263 PDF §3–5, 2026-09-23; MỘT tác giả; note hallberg_szabadvary_2024.md.</t>
+        </is>
+      </c>
+      <c r="L24" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-23; PMLR §3–5, Eq. (8)–(10), Tables 1–3</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="80" t="inlineStr">
+        <is>
+          <t>Lekeufack et al. 2023/2024 — Conformal Decision Theory</t>
+        </is>
+      </c>
+      <c r="B25" s="77" t="inlineStr">
+        <is>
+          <t>GẦN — direct decision-risk calibration (họ B)</t>
+        </is>
+      </c>
+      <c r="C25" s="77" t="inlineStr">
+        <is>
+          <t>Không age là biến chính</t>
+        </is>
+      </c>
+      <c r="D25" s="77" t="inlineStr">
+        <is>
+          <t>Empirical loss của executed decision</t>
+        </is>
+      </c>
+      <c r="E25" s="77" t="inlineStr">
+        <is>
+          <t>Không route top-2 margin</t>
+        </is>
+      </c>
+      <c r="F25" s="77" t="inlineStr">
+        <is>
+          <t>Có ví dụ nominal policy / safe backup</t>
+        </is>
+      </c>
+      <c r="G25" s="77" t="inlineStr">
+        <is>
+          <t>Theorem 1: average loss trên T bước ≤ ε+O(1/T) nếu eventually safe</t>
+        </is>
+      </c>
+      <c r="H25" s="77" t="inlineStr">
+        <is>
+          <t>Adversarial data sequence cho theorem, cần feedback loss</t>
+        </is>
+      </c>
+      <c r="I25" s="77" t="inlineStr">
+        <is>
+          <t>Robot navigation, trading, manufacturing</t>
+        </is>
+      </c>
+      <c r="J25" s="77" t="inlineStr">
+        <is>
+          <t>Không claim direct calibration của decision loss hoặc fallback là mới; không nhầm average risk với risk|ACCEPT.</t>
+        </is>
+      </c>
+      <c r="K25" s="77" t="inlineStr">
+        <is>
+          <t>ĐÃ KIỂM arXiv:2310.05921v3 §III–IV, Theorem 1 và đầu §V, 2026-09-23; note lekeufack_2024.md.</t>
+        </is>
+      </c>
+      <c r="L25" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-23; arXiv v3 §III–IV, Theorem 1, đầu §V</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="80" t="inlineStr">
+        <is>
+          <t>Gibbs &amp; Candès 2021 — ACI Under Distribution Shift</t>
+        </is>
+      </c>
+      <c r="B26" s="77" t="inlineStr">
+        <is>
+          <t>NỀN + baseline global ACI (họ E)</t>
+        </is>
+      </c>
+      <c r="C26" s="77" t="inlineStr">
+        <is>
+          <t>Không conditioning theo age</t>
+        </is>
+      </c>
+      <c r="D26" s="77" t="inlineStr">
+        <is>
+          <t>Online prediction coverage</t>
+        </is>
+      </c>
+      <c r="E26" s="77" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="F26" s="77" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="G26" s="77" t="inlineStr">
+        <is>
+          <t>Prop.4.1: time-average error lệch target O(1/(γT)) không cần exchangeability</t>
+        </is>
+      </c>
+      <c r="H26" s="77" t="inlineStr">
+        <is>
+          <t>Distribution shift bất kỳ cho Prop.4.1</t>
+        </is>
+      </c>
+      <c r="I26" s="77" t="inlineStr">
+        <is>
+          <t>Real datasets trong paper; chưa đối chiếu số</t>
+        </is>
+      </c>
+      <c r="J26" s="77" t="inlineStr">
+        <is>
+          <t>Global ACI phải là baseline; đo conditional age bins và selective risk riêng.</t>
+        </is>
+      </c>
+      <c r="K26" s="77" t="inlineStr">
+        <is>
+          <t>ĐÃ KIỂM arXiv:2106.00170 PDF §2, §4.1, Prop.4.1, 2026-09-23; note gibbs_candes_2021.md.</t>
+        </is>
+      </c>
+      <c r="L26" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-23; arXiv PDF §2, §4.1, Proposition 4.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="80" t="inlineStr">
+        <is>
+          <t>Ornee &amp; Sun 2021 — OU remote estimation through queues</t>
+        </is>
+      </c>
+      <c r="B27" s="77" t="inlineStr">
+        <is>
+          <t>NỀN — OU + AoI (họ D)</t>
+        </is>
+      </c>
+      <c r="C27" s="77" t="inlineStr">
+        <is>
+          <t>Có AoI, remote sampling</t>
+        </is>
+      </c>
+      <c r="D27" s="77" t="inlineStr">
+        <is>
+          <t>Estimation error / sampling policy</t>
+        </is>
+      </c>
+      <c r="E27" s="77" t="inlineStr">
+        <is>
+          <t>Không route ranking</t>
+        </is>
+      </c>
+      <c r="F27" s="77" t="inlineStr">
+        <is>
+          <t>Không action gate</t>
+        </is>
+      </c>
+      <c r="G27" s="77" t="inlineStr">
+        <is>
+          <t>Optimal threshold sampling dưới mô hình OU/queue</t>
+        </is>
+      </c>
+      <c r="H27" s="77" t="inlineStr">
+        <is>
+          <t>Stationary OU</t>
+        </is>
+      </c>
+      <c r="I27" s="77" t="inlineStr">
+        <is>
+          <t>Numerical comparison; chưa lấy số</t>
+        </is>
+      </c>
+      <c r="J27" s="77" t="inlineStr">
+        <is>
+          <t>Không claim quan hệ OU age và estimation error là mới; phân biệt state-level và decision-level.</t>
+        </is>
+      </c>
+      <c r="K27" s="77" t="inlineStr">
+        <is>
+          <t>ĐÃ KIỂM arXiv:1902.03552 abstract; PDF đã tải nhưng chưa đọc sâu, 2026-09-23; DOI 10.1109/TNET.2021.3078137.</t>
+        </is>
+      </c>
+      <c r="L27" s="35" t="inlineStr">
+        <is>
+          <t>Chưa xác định § đã đọc; cần đối chiếu trước khi dùng làm nguồn full text</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="80" t="inlineStr">
+        <is>
+          <t>Maatouk et al. 2020 — Age of Incorrect Information</t>
+        </is>
+      </c>
+      <c r="B28" s="77" t="inlineStr">
+        <is>
+          <t>NỀN — semantic freshness (họ D)</t>
+        </is>
+      </c>
+      <c r="C28" s="77" t="inlineStr">
+        <is>
+          <t>Có AoII; freshness gắn correctness</t>
+        </is>
+      </c>
+      <c r="D28" s="77" t="inlineStr">
+        <is>
+          <t>Status update quality</t>
+        </is>
+      </c>
+      <c r="E28" s="77" t="inlineStr">
+        <is>
+          <t>Không route ranking</t>
+        </is>
+      </c>
+      <c r="F28" s="77" t="inlineStr">
+        <is>
+          <t>Không route gate</t>
+        </is>
+      </c>
+      <c r="G28" s="77" t="inlineStr">
+        <is>
+          <t>CMDP/update policy; không conformal decision certificate</t>
+        </is>
+      </c>
+      <c r="H28" s="77" t="inlineStr">
+        <is>
+          <t>Markov source/status updates</t>
+        </is>
+      </c>
+      <c r="I28" s="77" t="inlineStr">
+        <is>
+          <t>Simulation; chưa lấy số</t>
+        </is>
+      </c>
+      <c r="J28" s="77" t="inlineStr">
+        <is>
+          <t>Không claim age cần xét correctness/task impact là mới.</t>
+        </is>
+      </c>
+      <c r="K28" s="77" t="inlineStr">
+        <is>
+          <t>ĐÃ KIỂM arXiv:1907.06604 abstract, 2026-09-23; DOI 10.1109/TNET.2020.3005549; bốn tác giả.</t>
+        </is>
+      </c>
+      <c r="L28" s="35" t="inlineStr">
+        <is>
+          <t>Chưa xác định § đã đọc; cần đối chiếu trước khi dùng làm nguồn full text</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="80" t="inlineStr">
+        <is>
+          <t>Qi et al. 2026 — Update for Decisions, Not Freshness</t>
+        </is>
+      </c>
+      <c r="B29" s="77" t="inlineStr">
+        <is>
+          <t>GẦN — stale remote state + selective edge offloading</t>
+        </is>
+      </c>
+      <c r="C29" s="77" t="inlineStr">
+        <is>
+          <t>Có: trạng thái remote cập nhật gián đoạn</t>
+        </is>
+      </c>
+      <c r="D29" s="77" t="inlineStr">
+        <is>
+          <t>Local / remote / reject user task, realized utility</t>
+        </is>
+      </c>
+      <c r="E29" s="77" t="inlineStr">
+        <is>
+          <t>Không route-cost top-2 margin theo abstract</t>
+        </is>
+      </c>
+      <c r="F29" s="77" t="inlineStr">
+        <is>
+          <t>Có gate–route/reject</t>
+        </is>
+      </c>
+      <c r="G29" s="77" t="inlineStr">
+        <is>
+          <t>RL/off-policy value learning, không conformal guarantee theo abstract</t>
+        </is>
+      </c>
+      <c r="H29" s="77" t="inlineStr">
+        <is>
+          <t>Asynchronous status update + decision</t>
+        </is>
+      </c>
+      <c r="I29" s="77" t="inlineStr">
+        <is>
+          <t>Abstract báo gains on-time completion 18.6–21.2%</t>
+        </is>
+      </c>
+      <c r="J29" s="77" t="inlineStr">
+        <is>
+          <t>Không claim kết hợp stale remote state với gate/reject là mới; khác biệt phải ở routing-cost risk và calibration.</t>
+        </is>
+      </c>
+      <c r="K29" s="77" t="inlineStr">
+        <is>
+          <t>Đã kiểm arXiv:2609.01082v1 metadata + abstract, 2026-09-23; full text chưa kiểm.</t>
+        </is>
+      </c>
+      <c r="L29" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; mới metadata/abstract, 2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="80" t="inlineStr">
+        <is>
+          <t>Tang et al. 2025 — Enhanced Route Planning with Calibrated Uncertainty Set</t>
+        </is>
+      </c>
+      <c r="B30" s="77" t="inlineStr">
+        <is>
+          <t>GẦN — conformal uncertainty + robust route planning</t>
+        </is>
+      </c>
+      <c r="C30" s="77" t="inlineStr">
+        <is>
+          <t>Chưa thấy age trong abstract</t>
+        </is>
+      </c>
+      <c r="D30" s="77" t="inlineStr">
+        <is>
+          <t>Route planning với uncertainty sets</t>
+        </is>
+      </c>
+      <c r="E30" s="77" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="F30" s="77" t="inlineStr">
+        <is>
+          <t>Không thấy abstention trong abstract</t>
+        </is>
+      </c>
+      <c r="G30" s="77" t="inlineStr">
+        <is>
+          <t>CQR-GAE conformal coverage + robust optimization</t>
+        </is>
+      </c>
+      <c r="H30" s="77" t="inlineStr">
+        <is>
+          <t>Chưa kiểm temporal dependence</t>
+        </is>
+      </c>
+      <c r="I30" s="77" t="inlineStr">
+        <is>
+          <t>Real-world traffic scenario theo abstract</t>
+        </is>
+      </c>
+      <c r="J30" s="77" t="inlineStr">
+        <is>
+          <t>Không claim conformal uncertainty cho route planning là mới; kiểm bản 2406.08281 do arXiv báo text overlap.</t>
+        </is>
+      </c>
+      <c r="K30" s="77" t="inlineStr">
+        <is>
+          <t>Đã kiểm arXiv:2503.10088v1 metadata + abstract, 2026-09-23; full text chưa kiểm; arXiv admin note: text overlap with 2406.08281.</t>
+        </is>
+      </c>
+      <c r="L30" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; mới metadata/abstract, 2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="83" t="inlineStr">
+        <is>
+          <t>Wang et al. 2026 — LEC: Selection-Conditioned Risk Control (arXiv:2512.01556v3)</t>
+        </is>
+      </c>
+      <c r="B31" s="83" t="inlineStr">
+        <is>
+          <t>RẤT GẦN ở trust target; model routing, không network path (họ F/B)</t>
+        </is>
+      </c>
+      <c r="C31" s="83" t="inlineStr">
+        <is>
+          <t>Không telemetry age</t>
+        </is>
+      </c>
+      <c r="D31" s="83" t="inlineStr">
+        <is>
+          <t>P(error | ACCEPT) ≤ α</t>
+        </is>
+      </c>
+      <c r="E31" s="83" t="inlineStr">
+        <is>
+          <t>Không route-cost top-2 margin</t>
+        </is>
+      </c>
+      <c r="F31" s="83" t="inlineStr">
+        <is>
+          <t>Có accept/abstain + delegate model</t>
+        </is>
+      </c>
+      <c r="G31" s="83" t="inlineStr">
+        <is>
+          <t>Finite-sample under exchangeability; E[S·err−αS]≤0</t>
+        </is>
+      </c>
+      <c r="H31" s="83" t="inlineStr">
+        <is>
+          <t>Exchangeability; chưa giải temporal OU dependence</t>
+        </is>
+      </c>
+      <c r="I31" s="83" t="inlineStr">
+        <is>
+          <t>QA/VQA model routing</t>
+        </is>
+      </c>
+      <c r="J31" s="83" t="inlineStr">
+        <is>
+          <t>Không claim selective risk|ACCEPT hay delegation guarantee là mới. So LEC-style gate cùng score age+margin và cùng calibration budget.</t>
+        </is>
+      </c>
+      <c r="K31" s="83" t="inlineStr">
+        <is>
+          <t>ĐÃ KIỂM arXiv v3 PDF §3, Thm 3.1–3.2, đầu §4 ngày 2026-09-23; proof/experiments chưa đọc hết. Note wang_lec_2026.md.</t>
+        </is>
+      </c>
+      <c r="L31" s="83" t="inlineStr">
+        <is>
+          <t>2026-09-23; arXiv v3 §3, Thm 3.1–3.2, đầu §4</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="84" t="inlineStr">
+        <is>
+          <t>Priye et al. 2026 — Available Guardrails (arXiv:2609.22048)</t>
+        </is>
+      </c>
+      <c r="B32" s="84" t="inlineStr">
+        <is>
+          <t>GẦN — finite-calibration feasibility cho selective risk (họ F/B)</t>
+        </is>
+      </c>
+      <c r="C32" s="84" t="inlineStr">
+        <is>
+          <t>Không telemetry age theo abstract</t>
+        </is>
+      </c>
+      <c r="D32" s="84" t="inlineStr">
+        <is>
+          <t>Selective certificate availability</t>
+        </is>
+      </c>
+      <c r="E32" s="84" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="F32" s="84" t="inlineStr">
+        <is>
+          <t>Có selective prediction</t>
+        </is>
+      </c>
+      <c r="G32" s="84" t="inlineStr">
+        <is>
+          <t>Finite-calibration feasibility; cần đọc theorem</t>
+        </is>
+      </c>
+      <c r="H32" s="84" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="I32" s="84" t="inlineStr">
+        <is>
+          <t>Metadata + abstract</t>
+        </is>
+      </c>
+      <c r="J32" s="84" t="inlineStr">
+        <is>
+          <t>Đánh giá sample size và ACCEPT rate khi thêm age bins; chưa dùng claim chi tiết từ full text.</t>
+        </is>
+      </c>
+      <c r="K32" s="84" t="inlineStr">
+        <is>
+          <t>Đã kiểm metadata/abstract arXiv ngày 2026-09-23; full text chưa đọc.</t>
+        </is>
+      </c>
+      <c r="L32" s="84" t="inlineStr">
+        <is>
+          <t>Chưa; mới metadata/abstract, 2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="83" t="inlineStr">
+        <is>
+          <t>Li et al. 2026 — From Freshness to Effectiveness (arXiv:2504.19507)</t>
+        </is>
+      </c>
+      <c r="B33" s="83" t="inlineStr">
+        <is>
+          <t>GẦN — age-aware remote decision (họ D)</t>
+        </is>
+      </c>
+      <c r="C33" s="83" t="inlineStr">
+        <is>
+          <t>Có age-aware decision</t>
+        </is>
+      </c>
+      <c r="D33" s="83" t="inlineStr">
+        <is>
+          <t>Remote decision effectiveness</t>
+        </is>
+      </c>
+      <c r="E33" s="83" t="inlineStr">
+        <is>
+          <t>Chưa kiểm route margin</t>
+        </is>
+      </c>
+      <c r="F33" s="83" t="inlineStr">
+        <is>
+          <t>Chưa kiểm gate</t>
+        </is>
+      </c>
+      <c r="G33" s="83" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="H33" s="83" t="inlineStr">
+        <is>
+          <t>Remote Markov decision process</t>
+        </is>
+      </c>
+      <c r="I33" s="83" t="inlineStr">
+        <is>
+          <t>Metadata + abstract</t>
+        </is>
+      </c>
+      <c r="J33" s="83" t="inlineStr">
+        <is>
+          <t>Không claim freshness-aware decision là mới; kiểm full text trước khi so với RQ1/RQ2.</t>
+        </is>
+      </c>
+      <c r="K33" s="83" t="inlineStr">
+        <is>
+          <t>Đã kiểm metadata/abstract 2026-09-23; DOI 10.1109/TIT.2026.3663678; note li_remote_decision_2026.md.</t>
+        </is>
+      </c>
+      <c r="L33" s="83" t="inlineStr">
+        <is>
+          <t>Chưa; mới metadata/abstract, 2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="35" t="inlineStr">
         <is>
           <t>DT4N candidate</t>
         </is>
       </c>
-      <c r="B22" s="35" t="inlineStr">
+      <c r="B34" s="35" t="inlineStr">
         <is>
           <t>Current research target</t>
         </is>
       </c>
-      <c r="C22" s="35" t="inlineStr">
+      <c r="C34" s="35" t="inlineStr">
         <is>
           <t>Có — telemetry age</t>
         </is>
       </c>
-      <c r="D22" s="35" t="inlineStr">
+      <c r="D34" s="35" t="inlineStr">
         <is>
           <t>Per-decision routing correctness / regret / SLA</t>
         </is>
       </c>
-      <c r="E22" s="35" t="inlineStr">
+      <c r="E34" s="35" t="inlineStr">
         <is>
           <t>Có — best-vs-second-best margin</t>
         </is>
       </c>
-      <c r="F22" s="35" t="inlineStr">
+      <c r="F34" s="35" t="inlineStr">
         <is>
           <t>Có — ACCEPT / ABSTAIN</t>
         </is>
       </c>
-      <c r="G22" s="35" t="inlineStr">
+      <c r="G34" s="35" t="inlineStr">
         <is>
           <t>Có — calibrated/conformal certificate</t>
         </is>
       </c>
-      <c r="H22" s="35" t="inlineStr">
+      <c r="H34" s="35" t="inlineStr">
         <is>
           <t>Block/time-aware evaluation planned/current</t>
         </is>
       </c>
-      <c r="I22" s="35" t="inlineStr">
+      <c r="I34" s="35" t="inlineStr">
         <is>
           <t>Simulator + Mininet; cần topology diversity</t>
         </is>
       </c>
-      <c r="J22" s="35" t="inlineStr">
-        <is>
-          <t>Candidate gap cần literature matrix xác nhận: age × margin → ranking risk + selective certification, not generic trust.</t>
-        </is>
-      </c>
-      <c r="K22" s="35" t="inlineStr">
-        <is>
-          <t>Claim đã thu hẹp sau khi cập nhật literature. KHÔNG claim: stale state → quyết định sai (Shaikh, Levin); chọn đường có tính bất định (Guérin–Orda); guarantee cho action được chọn (Kiyani, Zhu); conformal gate cho DT (OpenTwin v2); đưa AoI vào NDT (Zhu et al., link blockage); freshness metric cho DT (AoT, AoDT, AoS, EAP). CÒN LẠI (strong candidate): bản đồ risk age × margin cho từng quyết định trên vòng NDT emulated, kèm gate hiệu chỉnh. Baseline bắt buộc thêm: chọn đường theo xác suất kiểu Guérin–Orda, và forecast-to-now (AR(1)).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" s="54"/>
-    <row r="24" ht="48" customHeight="1" s="54">
-      <c r="A24" s="78" t="inlineStr">
-        <is>
-          <t>Chú thích: dòng tô vàng = paper thêm mới ngày 23/09/2026 (họ A: routing dưới trạng thái không chính xác; họ B: conformal → quyết định; họ C: giải pháp thay thế; họ D: freshness metric / NDT + AoI; 4 dòng cuối của họ D thêm sau khi đối chiếu một bản phân tích khác). Cột K = mức đã kiểm chứng và ưu tiên đọc. "Chưa kiểm" nghĩa là chưa đối chiếu với full text; không dùng các ô đó như fact khi viết paper.</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="n"/>
-      <c r="C24" s="1" t="n"/>
-      <c r="D24" s="1" t="n"/>
-      <c r="E24" s="1" t="n"/>
-      <c r="F24" s="1" t="n"/>
-      <c r="G24" s="1" t="n"/>
-      <c r="H24" s="1" t="n"/>
-      <c r="I24" s="1" t="n"/>
-      <c r="J24" s="1" t="n"/>
-      <c r="K24" s="1" t="n"/>
+      <c r="J34" s="35" t="inlineStr">
+        <is>
+          <t>Novelty chưa khóa: CERT đã có age-aware conformal route certificate và path gap; Hallberg Szabadváry đã có per-horizon ACI; CDT có direct decision-risk calibration. Cần chứng minh khác biệt age × top-2 margin → flip/harmful risk và lợi ích gate tại cùng budget trước DP1.</t>
+        </is>
+      </c>
+      <c r="K34" s="35" t="inlineStr">
+        <is>
+          <t>Cập nhật 2026-09-23 sau kill-search. Baselines bắt buộc cân nhắc: global ACI, per-age ACI, direct decision-risk controller, CERT-style age-widened route certificate, Guérin–Orda, forecast-to-now. Chưa được claim age+margin hoặc route certificate là mới cho đến khi kiểm CERT Appendix, Zhu và Guérin–Orda full text. Thêm Qi et al. 2026 và Tang et al. 2025 sau arXiv API search; mới kiểm abstract, không dùng làm kết luận full text.</t>
+        </is>
+      </c>
+      <c r="L34" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="L35" s="35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="78" t="inlineStr">
+        <is>
+          <t>Chú thích cập nhật 2026-09-23: cột L ghi chính xác phần PDF đã đối chiếu; trạng thái abstract/metadata không được tính là full text. LEC là đối thủ cho risk|ACCEPT; chưa kết luận DP1.</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="n"/>
+      <c r="C36" s="1" t="n"/>
+      <c r="D36" s="1" t="n"/>
+      <c r="E36" s="1" t="n"/>
+      <c r="F36" s="1" t="n"/>
+      <c r="G36" s="1" t="n"/>
+      <c r="H36" s="1" t="n"/>
+      <c r="I36" s="1" t="n"/>
+      <c r="J36" s="1" t="n"/>
+      <c r="K36" s="1" t="n"/>
+      <c r="L36" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A24:K24"/>
-  </mergeCells>
+  <autoFilter ref="A1:L34"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
P1/L1.8-L1.9: f05b rank agreement; full-text notes Burbano, Liyanage, Almohammedi, Fischer–Vöcking; positioning draft
</commit_message>
<xml_diff>
--- a/notes/01_literature/novelty_matrix.xlsx
+++ b/notes/01_literature/novelty_matrix.xlsx
@@ -2159,7 +2159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="54" min="1" max="1"/>
@@ -4306,6 +4306,254 @@
       <c r="L36" s="35" t="inlineStr">
         <is>
           <t>Không áp dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Burbano et al. 2025 — MO-HAN (arXiv:2511.10146v1)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Hàng xóm gần: dự đoán delay + hysteresis chọn edge server</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Không mô hình tuổi/nhiễu; dùng số đo thụ động mới nhất (§III-A, §IV-D)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Chọn edge server; latency E2E + tỉ lệ handover</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Có — S_j = α·T̂_j/T_max + (1−α)(1−R_j); đổi khi S_prev − S_best ≥ θ (Eq. 6–7, Alg. 1)</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Không (chỉ hysteresis trên điểm)</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Không; R_j = EWMA của chỉ báo 'latency ≤ (1+δ)·dự đoán' (Eq. 4–5)</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Tải nền ngẫu nhiên trên testbed; không mô hình động học tải</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Testbed thật, &gt;5000 mẫu, replay cùng dataset; NR/RR/LL-HAN; không CI (Table I)</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Không claim 'dự đoán + hysteresis' là mới. MO-HAN = ngưỡng tĩnh trên tâm có hiệu chỉnh; câu §IV-F và kết luận §V rộng hơn Table I (LL-HAN có mean, median thấp hơn)</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Đọc full text 2026-09-27 (AI soạn, tác giả kiểm)</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-09-27; §I–V, Alg. 1, Table I; Fig. 3–4 chỉ chú thích</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Liyanage et al. 2026 — Risk-aware stable server selection (arXiv:2604.21483v1; IWCMC 2026)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Hàng xóm gần nhất: (μ, σ) dự báo + hysteresis</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Không mô hình tuổi; cửa sổ trượt W quan sát gần nhất (§III-A)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Chọn edge server dưới SLO τ = 0,5 s; DMR, delay, tỉ lệ đổi</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Có — Score = μ + kσ; đổi khi cải thiện tương đối ≥ Δ trong N bước liên tiếp (Alg. 2)</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Có — feasibility: p_Norm &lt; ε và p_Cantelli &lt; ε (Alg. 1)</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Không; Normal surrogate + cận Cantelli (§III-B)</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Giả định dừng cục bộ trong cửa sổ (§III-D)</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Testbed 3 server, 1 client, một trace; không CI (Table II–III); replay 10 server minh hoạ (§V-F)</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Không claim 'dùng bất định + hysteresis' là mới. Khác: thiếu ô 'trung bình + hysteresis' nên không tách giá trị bất định; mục tiêu SLO ≠ mean-gain có ràng buộc harm; N ≥ 8 (không đổi) cho delay tốt nhất (Table III)</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Đọc full text 2026-09-27 (AI soạn, tác giả kiểm)</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-09-27; §I–VI, Alg. 1–2, Table I–III</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Almohammedi et al. 2026 — Twin-fidelity-aware xApp arbitration (arXiv:2607.22857v1; nộp IEEE TNSM)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Fallback theo độ tin cậy twin (cùng họ OpenTwin)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Không; drift = lệch có hệ thống d dB giữa twin và live (Eq. 6)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Chọn blend công suất phát; utility regret, QoS satisfaction</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Không margin; argmax Û (Eq. 11)</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Có — hard switch sang last-known-good khi EWMA |Û − U_live| ≥ τ (Eq. 12)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Không; công thức độ trễ phát hiện (Eq. 13)</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Môi trường dừng trong run (đường cong tính trước, §VI-B); A2 tối ưu biến chậm</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>MATLAB 5G, 7 cell, 20 seed, CI Student-t theo seed, so sánh paired (§VI-E)</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Không claim fallback theo fidelity toàn cục. Đề tài xét bất định TỪNG quyết định do tuổi/nhiễu, không phải lệch mô hình</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Đọc full text 2026-09-27 (AI soạn, tác giả kiểm)</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-09-27; §I–VIII, Alg. 1, Table I–V; hình chỉ chú thích</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Fischer &amp; Vöcking 2005/2009 — Adaptive routing with stale information (TR AIB-2005-06; PODC'05; TCS 410(36) 2009)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Nền lý thuyết: thông tin cũ gây dao động; luật đổi mềm</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Có — bulletin board cập nhật mỗi T (§1.3)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Hội tụ về cân bằng Wardrop / tránh dao động</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Migration μ không giảm theo chênh latency; α-smooth (§1.2)</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Có — hội tụ nếu T ≤ 1/(4Lαβ) (Lemma 1, Thm 1); dao động nếu T &gt; 8/(αβL) (Thm 3)</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Fluid limit; tải NỘI SINH (agent đổi đường làm đổi tải)</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Lý thuyết; ví dụ hai link (§2)</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Khác chế độ: đề tài = một luồng nhỏ, tải ngoại sinh (không herding). Không claim 'thông tin cũ làm luật tham lam hỏng/dao động'</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Đọc full text bản TR 2026-09-27 (AI soạn, tác giả kiểm); bản TCS 2009 chưa đối chiếu</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-09-27; TR 04/2005 §1–4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
P1/L1.9-L1.10: Seshadri–Katz full text; OpenAlex forward citation; DP1 per D18; F6 draft
</commit_message>
<xml_diff>
--- a/notes/01_literature/novelty_matrix.xlsx
+++ b/notes/01_literature/novelty_matrix.xlsx
@@ -2159,7 +2159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="54" min="1" max="1"/>
@@ -4554,6 +4554,68 @@
       <c r="L40" t="inlineStr">
         <is>
           <t>2026-09-27; TR 04/2005 §1–4</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Seshadri &amp; Katz 2003 — Dynamics of simultaneous overlay network routing (TR UCB/CSD-03-1291)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Hàng xóm gốc: hysteresis H trong đổi đường overlay tập thể</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Gián tiếp — thông tin lệch do luồng khác đổi trong cửa sổ đo + nhiễu đo 10% (§III–IV)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Mất gói trung bình của luồng overlay; số lần đổi</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Có — đổi khi băng thông đường tốt nhất &gt; hệ số H × đường hiện tại (§IV)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Không; mô phỏng mức luồng, 10 lần chạy, CI 95% (§III)</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Tải NỘI SINH (luồng overlay làm đổi tải); cross-traffic ngẫu nhiên</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Mô phỏng mức luồng, ~1000 luồng, 50 link, P_f = 25 (Fig. 1); quét H, IAT, P_f, T_r, cross-traffic</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Không claim 'H tối ưu phụ thuộc tham số' hay 'H thích nghi (MIMD)' là mới. Fig. 6: H cố định đủ khi luồng nhỏ — đề tài đo đúng chế độ này với oracle</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Đọc full text 2026-09-27 (AI soạn, tác giả kiểm)</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-09-27; §I–VII, Fig. 1–18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
P1v2/L1.10: literature khung mới — Jewson, Veeravalli–Kelly, Tiwari, Li (full text); Cisco AAR; mốc cổ điển; matrix v4; positioning v2 (nháp); DP1-v3 đề xuất
</commit_message>
<xml_diff>
--- a/notes/01_literature/novelty_matrix.xlsx
+++ b/notes/01_literature/novelty_matrix.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Conformal Tutorial 2022" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Novelty Matrix" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="All Papers Comparison" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Novelty Matrix v4" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Novelty Matrix'!$A$1:$L$34</definedName>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -78,8 +79,11 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -156,6 +160,11 @@
         <fgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border/>
@@ -164,7 +173,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -358,6 +367,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -822,6 +834,1112 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" style="54" min="1" max="1"/>
+    <col width="24" customWidth="1" style="54" min="2" max="2"/>
+    <col width="42" customWidth="1" style="54" min="3" max="3"/>
+    <col width="28" customWidth="1" style="54" min="4" max="4"/>
+    <col width="38" customWidth="1" style="54" min="5" max="5"/>
+    <col width="32" customWidth="1" style="54" min="6" max="6"/>
+    <col width="44" customWidth="1" style="54" min="7" max="7"/>
+    <col width="40" customWidth="1" style="54" min="8" max="8"/>
+    <col width="30" customWidth="1" style="54" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="85" t="inlineStr">
+        <is>
+          <t>Paper / Work</t>
+        </is>
+      </c>
+      <c r="B1" s="85" t="inlineStr">
+        <is>
+          <t>Họ / vai trò</t>
+        </is>
+      </c>
+      <c r="C1" s="85" t="inlineStr">
+        <is>
+          <t>Đo giá trị bất định so với ngưỡng đã tune?</t>
+        </is>
+      </c>
+      <c r="D1" s="85" t="inlineStr">
+        <is>
+          <t>Oracle cùng thông tin?</t>
+        </is>
+      </c>
+      <c r="E1" s="85" t="inlineStr">
+        <is>
+          <t>Cơ chế tạo bất định trực giao?</t>
+        </is>
+      </c>
+      <c r="F1" s="85" t="inlineStr">
+        <is>
+          <t>Phân rã thông tin / an toàn / thích nghi?</t>
+        </is>
+      </c>
+      <c r="G1" s="85" t="inlineStr">
+        <is>
+          <t>Khác biệt problem/method so với đề tài (D18)</t>
+        </is>
+      </c>
+      <c r="H1" s="85" t="inlineStr">
+        <is>
+          <t>Không được claim</t>
+        </is>
+      </c>
+      <c r="I1" s="85" t="inlineStr">
+        <is>
+          <t>Đã kiểm full text (ngày, §)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="35" t="inlineStr">
+        <is>
+          <t>DT4N v2 — đề tài (khung Phase 1 v2)</t>
+        </is>
+      </c>
+      <c r="B2" s="35" t="inlineStr">
+        <is>
+          <t>Đề tài</t>
+        </is>
+      </c>
+      <c r="C2" s="35" t="inlineStr">
+        <is>
+          <t>Có — K2(α) so với S0 / S0dir / SC trên cùng F, cùng α (F7 §2.3)</t>
+        </is>
+      </c>
+      <c r="D2" s="35" t="inlineStr">
+        <is>
+          <t>Có — oracle bin cùng F dọc quỹ đạo tham chiếu (K16); KHÔNG luôn là cận trên (F8: T10/FH −3,1 SE)</t>
+        </is>
+      </c>
+      <c r="E2" s="35" t="inlineStr">
+        <is>
+          <t>Sơ bộ — mức tải × độ cong (f05c ±26%); dị loại bị ngưỡng theo chiều hấp thụ (F7); lịch sử không tăng κ trong DES (F8, khám phá)</t>
+        </is>
+      </c>
+      <c r="F2" s="35" t="inlineStr">
+        <is>
+          <t>Có — thông tin 59–84% · an toàn 6–14% · tâm 1–4% · thuần ≤ 1,5% (F7 §3–4)</t>
+        </is>
+      </c>
+      <c r="G2" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H2" s="35" t="inlineStr">
+        <is>
+          <t>Nguyên lý đổi thứ tự và luật bậc hai (xem các dòng cổ điển)</t>
+        </is>
+      </c>
+      <c r="I2" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="35" t="inlineStr">
+        <is>
+          <t>Jewson 2003 — Moment based methods for ensemble assessment and calibration (arXiv:physics/0309042)</t>
+        </is>
+      </c>
+      <c r="B3" s="35" t="inlineStr">
+        <is>
+          <t>HỌ MỚI: dự báo tổ hợp — giá trị của spread</t>
+        </is>
+      </c>
+      <c r="C3" s="35" t="inlineStr">
+        <is>
+          <t>Gần nhất về khái niệm: chỉ-tâm (độ rộng hằng) vs tâm + spread, ngoài mẫu (§3, §4.4–4.5); thước đo likelihood, KHÔNG phải giá trị quyết định</t>
+        </is>
+      </c>
+      <c r="D3" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="E3" s="35" t="inlineStr">
+        <is>
+          <t>Một phần: COVS sau hiệu chỉnh nhỏ (§4.2); không cơ chế vật lý</t>
+        </is>
+      </c>
+      <c r="F3" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="G3" s="35" t="inlineStr">
+        <is>
+          <t>Problem: quyết định nhị phân có ngân sách harm (β ∝ λ); Method: oracle cùng thông tin + phân rã (đã kiểm full text)</t>
+        </is>
+      </c>
+      <c r="H3" s="35" t="inlineStr">
+        <is>
+          <t>'Độ rộng thêm ít khi biến thiên dự đoán được của bất định nhỏ; giá trị nằm ở tâm'</t>
+        </is>
+      </c>
+      <c r="I3" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-30; §1–5 (hình: chú thích)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="35" t="inlineStr">
+        <is>
+          <t>Houtekamer 1993 (MWR 121(6)); Whitaker &amp; Loughe 1998 (MWR 126)</t>
+        </is>
+      </c>
+      <c r="B4" s="35" t="inlineStr">
+        <is>
+          <t>Dự báo tổ hợp — spread–skill</t>
+        </is>
+      </c>
+      <c r="C4" s="35" t="inlineStr">
+        <is>
+          <t>Không trực tiếp: đo tương quan spread–skill</t>
+        </is>
+      </c>
+      <c r="D4" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="E4" s="35" t="inlineStr">
+        <is>
+          <t>Khái niệm: tương quan cực đại khi spread biến thiên mạnh (spread log-normal) ~ κ</t>
+        </is>
+      </c>
+      <c r="F4" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="G4" s="35" t="inlineStr">
+        <is>
+          <t>Chưa kiểm full text</t>
+        </is>
+      </c>
+      <c r="H4" s="35" t="inlineStr">
+        <is>
+          <t>'Giá trị bất định phụ thuộc độ phân tán của log s' là ý mới</t>
+        </is>
+      </c>
+      <c r="I4" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; abstract + thứ cấp 2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="35" t="inlineStr">
+        <is>
+          <t>Birge 1982 — Value of the stochastic solution (Math. Prog. 24(1):314–325)</t>
+        </is>
+      </c>
+      <c r="B5" s="35" t="inlineStr">
+        <is>
+          <t>Quy hoạch ngẫu nhiên — EVPI, VSS</t>
+        </is>
+      </c>
+      <c r="C5" s="35" t="inlineStr">
+        <is>
+          <t>Khái niệm: VSS = dùng phân phối vs cắm kỳ vọng (KHÔNG tune)</t>
+        </is>
+      </c>
+      <c r="D5" s="35" t="inlineStr">
+        <is>
+          <t>WS = thông tin hoàn hảo (không phải cùng thông tin)</t>
+        </is>
+      </c>
+      <c r="E5" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="F5" s="35" t="inlineStr">
+        <is>
+          <t>Hai bậc: EVPI (thông tin) + VSS (dùng phân phối)</t>
+        </is>
+      </c>
+      <c r="G5" s="35" t="inlineStr">
+        <is>
+          <t>Method: baseline đã tune; thêm bậc an toàn và tâm; oracle cùng thông tin — CHƯA kiểm full text Birge</t>
+        </is>
+      </c>
+      <c r="H5" s="35" t="inlineStr">
+        <is>
+          <t>Ý tưởng tách 'giá trị thông tin hoàn hảo' và 'giá trị dùng phân phối'</t>
+        </is>
+      </c>
+      <c r="I5" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; định nghĩa qua ≥ 3 nguồn thứ cấp 2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>von Winterfeldt &amp; Edwards 1973 — Flat maxima (TR 011313-4-T, U. Michigan)</t>
+        </is>
+      </c>
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>Toán cổ điển — flat maximum</t>
+        </is>
+      </c>
+      <c r="C6" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="D6" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="E6" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="F6" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="G6" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng (nền lý thuyết)</t>
+        </is>
+      </c>
+      <c r="H6" s="35" t="inlineStr">
+        <is>
+          <t>'Lệch gần tối ưu rẻ; tổn thất bậc hai'</t>
+        </is>
+      </c>
+      <c r="I6" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; thư mục 2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>Radner &amp; Stiglitz 1984; Chade &amp; Schlee 2002 (JET 107(2):421–452)</t>
+        </is>
+      </c>
+      <c r="B7" s="35" t="inlineStr">
+        <is>
+          <t>Toán cổ điển — giá trị biên thông tin = 0 tại 0</t>
+        </is>
+      </c>
+      <c r="C7" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="D7" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="E7" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="F7" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="G7" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng (nền lý thuyết)</t>
+        </is>
+      </c>
+      <c r="H7" s="35" t="inlineStr">
+        <is>
+          <t>'Giá trị thông tin nhỏ là bậc hai'</t>
+        </is>
+      </c>
+      <c r="I7" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; thư mục + abstract 2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="35" t="inlineStr">
+        <is>
+          <t>Mammen &amp; Tsybakov 1999; Audibert &amp; Tsybakov 2007 (AoS 35(2):608–633)</t>
+        </is>
+      </c>
+      <c r="B8" s="35" t="inlineStr">
+        <is>
+          <t>Toán cổ điển — điều kiện margin</t>
+        </is>
+      </c>
+      <c r="C8" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="D8" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="E8" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="F8" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="G8" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng (nền lý thuyết)</t>
+        </is>
+      </c>
+      <c r="H8" s="35" t="inlineStr">
+        <is>
+          <t>'Tổn thất ∝ mật độ gần biên × sai lệch²'</t>
+        </is>
+      </c>
+      <c r="I8" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; abstract 2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>Tiwari, Kar &amp; Tiwari 2026 — DT belief-state RL, latency-robust ISAC (arXiv:2604.25967v1)</t>
+        </is>
+      </c>
+      <c r="B9" s="35" t="inlineStr">
+        <is>
+          <t>DT dựng belief state từ telemetry trễ</t>
+        </is>
+      </c>
+      <c r="C9" s="35" t="inlineStr">
+        <is>
+          <t>Không; belief = ước lượng EKF (eq. 13)</t>
+        </is>
+      </c>
+      <c r="D9" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="E9" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="F9" s="35" t="inlineStr">
+        <is>
+          <t>Không; [I] DT-only 86% vs 88% ở 100 ms (§IV-D) ⇒ lợi ích chủ yếu ở tâm</t>
+        </is>
+      </c>
+      <c r="G9" s="35" t="inlineStr">
+        <is>
+          <t>Problem: hành động liên tục, không đổi/giữ, không ngân sách harm; Method: không oracle (đã kiểm)</t>
+        </is>
+      </c>
+      <c r="H9" s="35" t="inlineStr">
+        <is>
+          <t>'Twin dựng trạng thái hiện tại từ telemetry trễ để quyết định'</t>
+        </is>
+      </c>
+      <c r="I9" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-30; §I–V (hình: chú thích)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>Li, Wu, Lee &amp; Sun 2026 — From Freshness to Effectiveness (arXiv:2504.19507v3)</t>
+        </is>
+      </c>
+      <c r="B10" s="35" t="inlineStr">
+        <is>
+          <t>AoI/VoI cho quyết định từ xa</t>
+        </is>
+      </c>
+      <c r="C10" s="35" t="inlineStr">
+        <is>
+          <t>Không: so co-design với các chính sách lấy mẫu chuẩn (§VIII-A)</t>
+        </is>
+      </c>
+      <c r="D10" s="35" t="inlineStr">
+        <is>
+          <t>Không (MDP biết mô hình)</t>
+        </is>
+      </c>
+      <c r="E10" s="35" t="inlineStr">
+        <is>
+          <t>Không; tuổi là thông tin phụ trong thống kê đủ (Lemma 1)</t>
+        </is>
+      </c>
+      <c r="F10" s="35" t="inlineStr">
+        <is>
+          <t>Không; ngưỡng tần suất lấy mẫu (Thm 9, Cor. 2)</t>
+        </is>
+      </c>
+      <c r="G10" s="35" t="inlineStr">
+        <is>
+          <t>Problem: nguồn Markov hữu hạn, đồng thời chọn lấy mẫu; Method: không ngưỡng đã tune, không oracle cùng thông tin (đã kiểm)</t>
+        </is>
+      </c>
+      <c r="H10" s="35" t="inlineStr">
+        <is>
+          <t>'Tuổi là thông tin phụ cho quyết định'; 'độ tươi ≠ giá trị quyết định'</t>
+        </is>
+      </c>
+      <c r="I10" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-30; §I–VII; §VIII-A/B (hình: chú thích)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>Scherrer, Perrig &amp; Schmid 2020 — Value of Information in Selfish Routing (SIROCCO)</t>
+        </is>
+      </c>
+      <c r="B11" s="35" t="inlineStr">
+        <is>
+          <t>VoI trong định tuyến — tập thể (Wardrop)</t>
+        </is>
+      </c>
+      <c r="C11" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="D11" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="E11" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="F11" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="G11" s="35" t="inlineStr">
+        <is>
+          <t>Chế độ khác (tải nội sinh) — chưa kiểm full text</t>
+        </is>
+      </c>
+      <c r="H11" s="35" t="inlineStr">
+        <is>
+          <t>'Nhiều thông tin hơn có thể không giúp khi nhiều luồng cùng chọn đường'</t>
+        </is>
+      </c>
+      <c r="I11" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; abstract 2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="35" t="inlineStr">
+        <is>
+          <t>Keralapura, Chuah, Taft &amp; Iannaccone 2008 — Race conditions in coexisting overlays (ToN 16(1))</t>
+        </is>
+      </c>
+      <c r="B12" s="35" t="inlineStr">
+        <is>
+          <t>Dao động nhiều overlay — tập thể</t>
+        </is>
+      </c>
+      <c r="C12" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="D12" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="E12" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="F12" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="G12" s="35" t="inlineStr">
+        <is>
+          <t>Chế độ khác (nhiều overlay) — chưa kiểm full text</t>
+        </is>
+      </c>
+      <c r="H12" s="35" t="inlineStr">
+        <is>
+          <t>'Nhiều bộ chọn đường độc lập có thể đồng bộ và dao động'</t>
+        </is>
+      </c>
+      <c r="I12" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; abstract/đoạn trích 2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="35" t="inlineStr">
+        <is>
+          <t>Seshadri &amp; Katz 2003 — Dynamics of simultaneous overlay network routing (TR; WIRED)</t>
+        </is>
+      </c>
+      <c r="B13" s="35" t="inlineStr">
+        <is>
+          <t>Hysteresis H, overlay tập thể</t>
+        </is>
+      </c>
+      <c r="C13" s="35" t="inlineStr">
+        <is>
+          <t>Không trực tiếp: quét H cố định, MIMD-H, ngẫu nhiên hoá (§IV–V)</t>
+        </is>
+      </c>
+      <c r="D13" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="E13" s="35" t="inlineStr">
+        <is>
+          <t>Gián tiếp: H tối ưu phụ thuộc tham số (Fig. 4–5)</t>
+        </is>
+      </c>
+      <c r="F13" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="G13" s="35" t="inlineStr">
+        <is>
+          <t>Problem: tập thể, metric mất gói; Method: không oracle (đã kiểm 27/09)</t>
+        </is>
+      </c>
+      <c r="H13" s="35" t="inlineStr">
+        <is>
+          <t>'H tối ưu phụ thuộc tham số'; 'H thích nghi (MIMD)'</t>
+        </is>
+      </c>
+      <c r="I13" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-27; §I–VII</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="35" t="inlineStr">
+        <is>
+          <t>Fischer &amp; Vöcking 2005/2009 — Adaptive routing with stale information</t>
+        </is>
+      </c>
+      <c r="B14" s="35" t="inlineStr">
+        <is>
+          <t>Thông tin cũ gây dao động (tập thể)</t>
+        </is>
+      </c>
+      <c r="C14" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="D14" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="E14" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="F14" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="G14" s="35" t="inlineStr">
+        <is>
+          <t>Problem: tải nội sinh, fluid limit (đã kiểm 27/09)</t>
+        </is>
+      </c>
+      <c r="H14" s="35" t="inlineStr">
+        <is>
+          <t>'Thông tin cũ làm luật tham lam dao động'</t>
+        </is>
+      </c>
+      <c r="I14" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-27; TR §1–4</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="35" t="inlineStr">
+        <is>
+          <t>Liyanage et al. 2026 — Risk-aware stable server selection (arXiv:2604.21483v1)</t>
+        </is>
+      </c>
+      <c r="B15" s="35" t="inlineStr">
+        <is>
+          <t>(μ, σ) + hysteresis</t>
+        </is>
+      </c>
+      <c r="C15" s="35" t="inlineStr">
+        <is>
+          <t>Không tách được: thiếu ô 'trung bình + hysteresis' (Table II); một trace, không CI</t>
+        </is>
+      </c>
+      <c r="D15" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="E15" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="F15" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="G15" s="35" t="inlineStr">
+        <is>
+          <t>Problem: SLO, không ngân sách harm; Method: không oracle, không factorial (đã kiểm 27/09)</t>
+        </is>
+      </c>
+      <c r="H15" s="35" t="inlineStr">
+        <is>
+          <t>'Dùng bất định + hysteresis để chọn đích'</t>
+        </is>
+      </c>
+      <c r="I15" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-27; §I–VI</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>Burbano et al. 2025 — MO-HAN (arXiv:2511.10146v1)</t>
+        </is>
+      </c>
+      <c r="B16" s="35" t="inlineStr">
+        <is>
+          <t>Dự đoán + hysteresis</t>
+        </is>
+      </c>
+      <c r="C16" s="35" t="inlineStr">
+        <is>
+          <t>Không: hysteresis trên điểm có hiệu chỉnh (Eq. 4–7)</t>
+        </is>
+      </c>
+      <c r="D16" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="E16" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="F16" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="G16" s="35" t="inlineStr">
+        <is>
+          <t>Problem: không tuổi/nhiễu; Method: không oracle, không CI (đã kiểm 27/09)</t>
+        </is>
+      </c>
+      <c r="H16" s="35" t="inlineStr">
+        <is>
+          <t>'Dự đoán + hysteresis'</t>
+        </is>
+      </c>
+      <c r="I16" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-27; §I–V</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="35" t="inlineStr">
+        <is>
+          <t>Almohammedi et al. 2026 — Twin-fidelity-aware xApp arbitration (arXiv:2607.22857v1)</t>
+        </is>
+      </c>
+      <c r="B17" s="35" t="inlineStr">
+        <is>
+          <t>Fallback theo fidelity twin</t>
+        </is>
+      </c>
+      <c r="C17" s="35" t="inlineStr">
+        <is>
+          <t>Không: fallback khi EWMA sai số ≥ τ (Eq. 12)</t>
+        </is>
+      </c>
+      <c r="D17" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="E17" s="35" t="inlineStr">
+        <is>
+          <t>Không (drift toàn cục)</t>
+        </is>
+      </c>
+      <c r="F17" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="G17" s="35" t="inlineStr">
+        <is>
+          <t>Problem: lệch mô hình toàn cục (đã kiểm 27/09)</t>
+        </is>
+      </c>
+      <c r="H17" s="35" t="inlineStr">
+        <is>
+          <t>'Fallback theo fidelity twin'</t>
+        </is>
+      </c>
+      <c r="I17" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-27; §I–VIII</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="35" t="inlineStr">
+        <is>
+          <t>OpenTwin v2 2026 (arXiv:2605.24662v2)</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="inlineStr">
+        <is>
+          <t>Cổng an toàn hành động cho DT</t>
+        </is>
+      </c>
+      <c r="C18" s="35" t="inlineStr">
+        <is>
+          <t>Không: gate an toàn tuyệt đối C_t(a) ⊆ S (§VI)</t>
+        </is>
+      </c>
+      <c r="D18" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="E18" s="35" t="inlineStr">
+        <is>
+          <t>Không (drift qua hiệu chỉnh trực tuyến)</t>
+        </is>
+      </c>
+      <c r="F18" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="G18" s="35" t="inlineStr">
+        <is>
+          <t>Problem: an toàn một hành động (đã kiểm 23/09)</t>
+        </is>
+      </c>
+      <c r="H18" s="35" t="inlineStr">
+        <is>
+          <t>'Cổng tin cậy/conformal cho DT'</t>
+        </is>
+      </c>
+      <c r="I18" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-23; §V–VIII</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="35" t="inlineStr">
+        <is>
+          <t>CERT 2026; LEC 2026; Zhu et al. 2026; Lekeufack et al. 2024 (chi tiết: sheet v3)</t>
+        </is>
+      </c>
+      <c r="B19" s="35" t="inlineStr">
+        <is>
+          <t>Gate/certificate cho quyết định (RQ2 cũ)</t>
+        </is>
+      </c>
+      <c r="C19" s="35" t="inlineStr">
+        <is>
+          <t>Không: hiệu chỉnh rủi ro của gate</t>
+        </is>
+      </c>
+      <c r="D19" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="E19" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="F19" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="G19" s="35" t="inlineStr">
+        <is>
+          <t>Trùng một phần gate/luật — lý do DP1 = NARROW (F6)</t>
+        </is>
+      </c>
+      <c r="H19" s="35" t="inlineStr">
+        <is>
+          <t>Xem v3</t>
+        </is>
+      </c>
+      <c r="I19" s="35" t="inlineStr">
+        <is>
+          <t>Xem v3 (23/09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="35" t="inlineStr">
+        <is>
+          <t>Veeravalli &amp; Kelly 1997 — A locally optimal handoff algorithm (IEEE TVT 46(3):603–609)</t>
+        </is>
+      </c>
+      <c r="B20" s="35" t="inlineStr">
+        <is>
+          <t>HỌ HANDOVER — luật so xác suất vs hysteresis đã tune</t>
+        </is>
+      </c>
+      <c r="C20" s="35" t="inlineStr">
+        <is>
+          <t>CÓ, gần nhất: LO vs hysteresis và hysteresis-threshold (2 tham số) trên CÙNG bộ dự báo, cùng số handoff; LO ≈ hysteresis-threshold tốt nhất (§V, Fig. 3)</t>
+        </is>
+      </c>
+      <c r="D20" s="35" t="inlineStr">
+        <is>
+          <t>Không cùng thông tin: DP tối ưu biết trước quỹ đạo, dùng làm mốc (§III, Fig. 3)</t>
+        </is>
+      </c>
+      <c r="E20" s="35" t="inlineStr">
+        <is>
+          <t>Không: phương sai có điều kiện không phụ thuộc vị trí (§IV) ⇒ κ = 0 theo cấu trúc; lợi thế LO đến từ phụ thuộc mức tín hiệu</t>
+        </is>
+      </c>
+      <c r="F20" s="35" t="inlineStr">
+        <is>
+          <t>Không; dự báo tốt hơn (tốc độ chậm) làm LO lợi hơn hysteresis (Fig. 4–5)</t>
+        </is>
+      </c>
+      <c r="G20" s="35" t="inlineStr">
+        <is>
+          <t>Method: tách kênh độ rộng (K2 − SC) khi κ &gt; 0 — V–K không làm được vì phương sai hằng; phân rã; oracle một bước cùng thông tin. Problem: delay hàng đợi dưới telemetry cũ + nhiễu (đã kiểm full text)</t>
+        </is>
+      </c>
+      <c r="H20" s="35" t="inlineStr">
+        <is>
+          <t>'So luật dùng xác suất với luật tĩnh đã tune, cùng dự báo, cùng ngân sách'; 'luật dựa mô hình thích nghi môi trường tốt hơn hysteresis cố định'; tương đương ràng buộc–Bayes</t>
+        </is>
+      </c>
+      <c r="I20" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-30; §I–VI + Phụ lục</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="35" t="inlineStr">
+        <is>
+          <t>Cisco SD-WAN Policies Config Guide vEdge 20.x — chương Application-Aware Routing</t>
+        </is>
+      </c>
+      <c r="B21" s="35" t="inlineStr">
+        <is>
+          <t>Nguồn thực tế SD-WAN (tài liệu nhà cung cấp)</t>
+        </is>
+      </c>
+      <c r="C21" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="D21" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="E21" s="35" t="inlineStr">
+        <is>
+          <t>Telemetry thực: BFD 1 s trên MỌI tunnel; trung bình poll 10 phút; SLA trên 6 poll (1 giờ) — để damping</t>
+        </is>
+      </c>
+      <c r="F21" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="G21" s="35" t="inlineStr">
+        <is>
+          <t>Luật thực tế = ngưỡng SLA tuyệt đối trên trung bình dài + dải variance + tunnel dampening — đúng họ 'tĩnh + damping' đề tài dùng làm baseline</t>
+        </is>
+      </c>
+      <c r="H21" s="35" t="inlineStr">
+        <is>
+          <t>Không dùng 'SD-WAN đo path phụ thưa hơn' cho cấu hình mặc định</t>
+        </is>
+      </c>
+      <c r="I21" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-30; toàn chương (HTML)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="35" t="inlineStr">
+        <is>
+          <t>Richardson 2000 — Skill and relative economic value of the ECMWF EPS (QJRMS 126:649–667); Murphy 1977</t>
+        </is>
+      </c>
+      <c r="B22" s="35" t="inlineStr">
+        <is>
+          <t>Giá trị kinh tế của dự báo — cost–loss, REV</t>
+        </is>
+      </c>
+      <c r="C22" s="35" t="inlineStr">
+        <is>
+          <t>Một phần: xác suất EPS vs dự báo tất định cùng mô hình (abstract); có tune ngưỡng tất định không — chưa kiểm</t>
+        </is>
+      </c>
+      <c r="D22" s="35" t="inlineStr">
+        <is>
+          <t>Chuẩn hoá theo dự báo hoàn hảo (thông tin hoàn hảo, không cùng thông tin)</t>
+        </is>
+      </c>
+      <c r="E22" s="35" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="F22" s="35" t="inlineStr">
+        <is>
+          <t>Không (một tỉ lệ REV)</t>
+        </is>
+      </c>
+      <c r="G22" s="35" t="inlineStr">
+        <is>
+          <t>Method: phân rã bốn bậc + baseline tâm đã tune — chưa kiểm full text Richardson</t>
+        </is>
+      </c>
+      <c r="H22" s="35" t="inlineStr">
+        <is>
+          <t>'Chuẩn hoá giá trị quyết định theo thông tin hoàn hảo' (tỉ lệ headroom ~ REV)</t>
+        </is>
+      </c>
+      <c r="I22" s="35" t="inlineStr">
+        <is>
+          <t>Chưa; abstract + định nghĩa REV qua ≥ 3 nguồn thứ cấp 2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="35" t="inlineStr">
+        <is>
+          <t>Tài liệu Linux kernel — MPTCP sysctl stale_loss_cnt</t>
+        </is>
+      </c>
+      <c r="B23" s="35" t="inlineStr">
+        <is>
+          <t>Nguồn thực tế (ĐÍNH CHÍNH L1.8)</t>
+        </is>
+      </c>
+      <c r="C23" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="D23" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="E23" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="F23" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="G23" s="35" t="inlineStr">
+        <is>
+          <t>Không áp dụng</t>
+        </is>
+      </c>
+      <c r="H23" s="35" t="inlineStr">
+        <is>
+          <t>Không dùng 'MPTCP stale subflow' làm bằng chứng path phụ đo thưa: 'stale' = subflow không tiến triển, scheduler bỏ qua</t>
+        </is>
+      </c>
+      <c r="I23" s="35" t="inlineStr">
+        <is>
+          <t>2026-09-30; tài liệu gốc (docs.kernel.org)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>